<commit_message>
chore: save user template changes
</commit_message>
<xml_diff>
--- a/METRADO_PLANTILLA_5.xlsx
+++ b/METRADO_PLANTILLA_5.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DEDBFF0-72A5-447C-BB69-2EB7CE7B7B82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB1C214E-7327-4962-A689-3CA59CB7B9E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -735,7 +735,7 @@
     <numFmt numFmtId="169" formatCode="dd/mm/yyyy&quot;  &quot;hh&quot;:&quot;mm&quot;:&quot;ss\ AM/PM"/>
     <numFmt numFmtId="170" formatCode="dd/mm/yy;@"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -903,6 +903,12 @@
       <name val="Arial Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="8"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -1044,7 +1050,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="149">
+  <cellXfs count="150">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1429,6 +1435,9 @@
     </xf>
     <xf numFmtId="2" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="26" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -30412,7 +30421,7 @@
     <col min="23" max="23" width="8" style="25" customWidth="1"/>
     <col min="24" max="24" width="5.796875" style="25" customWidth="1"/>
     <col min="25" max="25" width="10.3984375" customWidth="1"/>
-    <col min="26" max="26" width="32.3984375" customWidth="1"/>
+    <col min="26" max="26" width="49.59765625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -30745,7 +30754,7 @@
       <c r="Q10" s="87"/>
       <c r="R10" s="87"/>
       <c r="S10" s="87"/>
-      <c r="T10" s="87"/>
+      <c r="T10" s="149"/>
       <c r="U10" s="87"/>
       <c r="V10" s="84"/>
       <c r="W10" s="38"/>

</xml_diff>

<commit_message>
chore: save state before unifying liquidaciones interface
</commit_message>
<xml_diff>
--- a/METRADO_PLANTILLA_5.xlsx
+++ b/METRADO_PLANTILLA_5.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CB753F4-05E6-4EB4-84FC-AA6BC3F01C74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
@@ -732,8 +732,8 @@
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dddd\,\ yyyy"/>
     <numFmt numFmtId="165" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="168" formatCode="#,##0.00_);\-#,##0.00"/>
-    <numFmt numFmtId="169" formatCode="dd/mm/yyyy&quot;  &quot;hh&quot;:&quot;mm&quot;:&quot;ss\ AM/PM"/>
+    <numFmt numFmtId="166" formatCode="#,##0.00_);\-#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="dd/mm/yyyy&quot;  &quot;hh&quot;:&quot;mm&quot;:&quot;ss\ AM/PM"/>
   </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
@@ -1124,16 +1124,16 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="10" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1141,6 +1141,45 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="11" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="11" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1164,45 +1203,6 @@
     <xf numFmtId="2" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="10" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="10" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="10" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="10" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="11" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="11" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1214,10 +1214,74 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color auto="1"/>
+        <name val="Arial Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="hair">
+          <color rgb="FF000000"/>
+        </left>
+        <right/>
+        <top style="hair">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="hair">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="8"/>
-        <color rgb="FFC00000"/>
+        <color auto="1"/>
+        <name val="Arial Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="hair">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="hair">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="hair">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="hair">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color auto="1"/>
         <name val="Arial Narrow"/>
         <family val="2"/>
         <scheme val="none"/>
@@ -1239,12 +1303,14 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
+        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="8"/>
-        <color auto="1"/>
+        <color rgb="FFC00000"/>
         <name val="Arial Narrow"/>
         <family val="2"/>
         <scheme val="none"/>
@@ -1319,72 +1385,6 @@
         <bottom style="hair">
           <color rgb="FF000000"/>
         </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color auto="1"/>
-        <name val="Arial Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="hair">
-          <color rgb="FF000000"/>
-        </left>
-        <right/>
-        <top style="hair">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="hair">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color auto="1"/>
-        <name val="Arial Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="hair">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="hair">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="hair">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="hair">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -2026,6 +2026,15 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
       <border outline="0">
         <left style="hair">
           <color rgb="FF000000"/>
@@ -2040,15 +2049,6 @@
           <color rgb="FF000000"/>
         </bottom>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <color auto="1"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -2161,7 +2161,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table_1" displayName="Table_1" ref="B7:AA419" headerRowCount="0" headerRowDxfId="28" totalsRowDxfId="27" tableBorderDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table_1" displayName="Table_1" ref="B7:AA419" headerRowCount="0" headerRowDxfId="28" totalsRowDxfId="26" tableBorderDxfId="27">
   <tableColumns count="26">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="GRADO" dataDxfId="25"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="FECHA" dataDxfId="24"/>
@@ -2183,12 +2183,12 @@
     <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="PARCIAL" dataDxfId="8"/>
     <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="N° VECES" dataDxfId="7"/>
     <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="ACERO" dataDxfId="6"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="TOTAL" dataDxfId="3"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="TOTAL 2" dataDxfId="2"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="UNIDAD" dataDxfId="0"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="MODIF." dataDxfId="1"/>
-    <tableColumn id="25" xr3:uid="{3865C319-53D6-41C8-9C4C-31FA4F4E0948}" name="Columna1" dataDxfId="5"/>
-    <tableColumn id="26" xr3:uid="{F0183D40-AE54-4413-976E-0B00C7B637A5}" name="Columna2" dataDxfId="4"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="TOTAL" dataDxfId="5"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="TOTAL 2" dataDxfId="4"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="UNIDAD" dataDxfId="3"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="MODIF." dataDxfId="2"/>
+    <tableColumn id="25" xr3:uid="{3865C319-53D6-41C8-9C4C-31FA4F4E0948}" name="Columna1" dataDxfId="1"/>
+    <tableColumn id="26" xr3:uid="{F0183D40-AE54-4413-976E-0B00C7B637A5}" name="Columna2" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2418,19 +2418,19 @@
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
-      <c r="H1" s="42" t="s">
+      <c r="H1" s="55" t="s">
         <v>0</v>
       </c>
-      <c r="I1" s="43"/>
-      <c r="J1" s="43"/>
-      <c r="K1" s="43"/>
-      <c r="L1" s="43"/>
-      <c r="M1" s="43"/>
-      <c r="N1" s="43"/>
-      <c r="O1" s="43"/>
-      <c r="P1" s="43"/>
-      <c r="Q1" s="43"/>
-      <c r="R1" s="43"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
+      <c r="P1" s="56"/>
+      <c r="Q1" s="56"/>
+      <c r="R1" s="56"/>
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
       <c r="U1" s="1"/>
@@ -2500,25 +2500,25 @@
     </row>
     <row r="4" spans="1:26" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
-      <c r="B4" s="44">
+      <c r="B4" s="57">
         <v>45809</v>
       </c>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="45"/>
-      <c r="G4" s="45"/>
-      <c r="H4" s="45"/>
-      <c r="I4" s="45"/>
-      <c r="J4" s="45"/>
-      <c r="K4" s="45"/>
-      <c r="L4" s="45"/>
-      <c r="M4" s="45"/>
-      <c r="N4" s="45"/>
-      <c r="O4" s="45"/>
-      <c r="P4" s="45"/>
-      <c r="Q4" s="45"/>
-      <c r="R4" s="45"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
+      <c r="G4" s="58"/>
+      <c r="H4" s="58"/>
+      <c r="I4" s="58"/>
+      <c r="J4" s="58"/>
+      <c r="K4" s="58"/>
+      <c r="L4" s="58"/>
+      <c r="M4" s="58"/>
+      <c r="N4" s="58"/>
+      <c r="O4" s="58"/>
+      <c r="P4" s="58"/>
+      <c r="Q4" s="58"/>
+      <c r="R4" s="58"/>
       <c r="S4" s="1"/>
       <c r="T4" s="1"/>
       <c r="U4" s="1"/>
@@ -2530,38 +2530,38 @@
     </row>
     <row r="5" spans="1:26" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
-      <c r="B5" s="49" t="s">
+      <c r="B5" s="62" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="51" t="s">
+      <c r="C5" s="64" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="49" t="s">
+      <c r="D5" s="62" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="52" t="s">
+      <c r="E5" s="65" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="52" t="s">
+      <c r="F5" s="65" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="52" t="s">
+      <c r="G5" s="65" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="52" t="s">
+      <c r="H5" s="65" t="s">
         <v>8</v>
       </c>
-      <c r="I5" s="52" t="s">
+      <c r="I5" s="65" t="s">
         <v>9</v>
       </c>
-      <c r="J5" s="46" t="s">
+      <c r="J5" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="K5" s="47"/>
-      <c r="L5" s="47"/>
-      <c r="M5" s="47"/>
-      <c r="N5" s="47"/>
-      <c r="O5" s="48"/>
+      <c r="K5" s="60"/>
+      <c r="L5" s="60"/>
+      <c r="M5" s="60"/>
+      <c r="N5" s="60"/>
+      <c r="O5" s="61"/>
       <c r="P5" s="4"/>
       <c r="Q5" s="5"/>
       <c r="R5" s="6"/>
@@ -2576,14 +2576,14 @@
     </row>
     <row r="6" spans="1:26" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
-      <c r="B6" s="50"/>
-      <c r="C6" s="50"/>
-      <c r="D6" s="50"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="50"/>
-      <c r="G6" s="50"/>
-      <c r="H6" s="50"/>
-      <c r="I6" s="50"/>
+      <c r="B6" s="63"/>
+      <c r="C6" s="63"/>
+      <c r="D6" s="63"/>
+      <c r="E6" s="63"/>
+      <c r="F6" s="63"/>
+      <c r="G6" s="63"/>
+      <c r="H6" s="63"/>
+      <c r="I6" s="63"/>
       <c r="J6" s="7" t="s">
         <v>11</v>
       </c>
@@ -30782,1934 +30782,1934 @@
     <col min="28" max="16384" width="12.69921875" style="40"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="59" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:27" s="48" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="41"/>
-      <c r="B1" s="58"/>
-      <c r="C1" s="58"/>
-      <c r="D1" s="58"/>
-      <c r="E1" s="58"/>
-      <c r="F1" s="58"/>
-      <c r="G1" s="58"/>
-      <c r="H1" s="58"/>
-      <c r="I1" s="58"/>
-      <c r="J1" s="58"/>
-      <c r="K1" s="58"/>
-      <c r="L1" s="58"/>
-      <c r="M1" s="58"/>
-      <c r="N1" s="58"/>
-      <c r="O1" s="58"/>
-      <c r="P1" s="58"/>
-      <c r="Q1" s="58"/>
-      <c r="R1" s="58"/>
-      <c r="S1" s="58"/>
-      <c r="T1" s="58"/>
-      <c r="U1" s="58"/>
-      <c r="V1" s="58"/>
-      <c r="W1" s="64"/>
-      <c r="X1" s="64"/>
-      <c r="Y1" s="58"/>
-      <c r="Z1" s="58" t="s">
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
+      <c r="L1" s="47"/>
+      <c r="M1" s="47"/>
+      <c r="N1" s="47"/>
+      <c r="O1" s="47"/>
+      <c r="P1" s="47"/>
+      <c r="Q1" s="47"/>
+      <c r="R1" s="47"/>
+      <c r="S1" s="47"/>
+      <c r="T1" s="47"/>
+      <c r="U1" s="47"/>
+      <c r="V1" s="47"/>
+      <c r="W1" s="53"/>
+      <c r="X1" s="53"/>
+      <c r="Y1" s="47"/>
+      <c r="Z1" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="AA1" s="58"/>
+      <c r="AA1" s="47"/>
     </row>
     <row r="2" spans="1:27" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="I2" s="58"/>
-      <c r="J2" s="58"/>
-      <c r="K2" s="58"/>
-      <c r="L2" s="58"/>
-      <c r="M2" s="58"/>
-      <c r="N2" s="58"/>
-      <c r="O2" s="58"/>
-      <c r="P2" s="58"/>
-      <c r="Q2" s="58"/>
-      <c r="R2" s="58"/>
-      <c r="S2" s="58"/>
-      <c r="T2" s="58"/>
-      <c r="U2" s="58"/>
-      <c r="V2" s="58"/>
-      <c r="W2" s="64"/>
-      <c r="X2" s="64"/>
-      <c r="Y2" s="58"/>
-      <c r="Z2" s="58" t="s">
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+      <c r="L2" s="47"/>
+      <c r="M2" s="47"/>
+      <c r="N2" s="47"/>
+      <c r="O2" s="47"/>
+      <c r="P2" s="47"/>
+      <c r="Q2" s="47"/>
+      <c r="R2" s="47"/>
+      <c r="S2" s="47"/>
+      <c r="T2" s="47"/>
+      <c r="U2" s="47"/>
+      <c r="V2" s="47"/>
+      <c r="W2" s="53"/>
+      <c r="X2" s="53"/>
+      <c r="Y2" s="47"/>
+      <c r="Z2" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="AA2" s="58"/>
+      <c r="AA2" s="47"/>
     </row>
     <row r="3" spans="1:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="58"/>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
-      <c r="I3" s="58"/>
-      <c r="J3" s="58"/>
-      <c r="K3" s="58"/>
-      <c r="L3" s="58"/>
-      <c r="M3" s="58"/>
-      <c r="N3" s="58"/>
-      <c r="O3" s="58"/>
-      <c r="P3" s="58"/>
-      <c r="Q3" s="58"/>
-      <c r="R3" s="58"/>
-      <c r="S3" s="58"/>
-      <c r="T3" s="58"/>
-      <c r="U3" s="58"/>
-      <c r="V3" s="58"/>
-      <c r="W3" s="64"/>
-      <c r="X3" s="64"/>
-      <c r="Y3" s="58"/>
-      <c r="Z3" s="58"/>
-      <c r="AA3" s="58"/>
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
+      <c r="I3" s="47"/>
+      <c r="J3" s="47"/>
+      <c r="K3" s="47"/>
+      <c r="L3" s="47"/>
+      <c r="M3" s="47"/>
+      <c r="N3" s="47"/>
+      <c r="O3" s="47"/>
+      <c r="P3" s="47"/>
+      <c r="Q3" s="47"/>
+      <c r="R3" s="47"/>
+      <c r="S3" s="47"/>
+      <c r="T3" s="47"/>
+      <c r="U3" s="47"/>
+      <c r="V3" s="47"/>
+      <c r="W3" s="53"/>
+      <c r="X3" s="53"/>
+      <c r="Y3" s="47"/>
+      <c r="Z3" s="47"/>
+      <c r="AA3" s="47"/>
     </row>
     <row r="4" spans="1:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="59" t="s">
+      <c r="B4" s="48" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="58"/>
-      <c r="D4" s="58"/>
-      <c r="E4" s="58"/>
-      <c r="F4" s="58"/>
-      <c r="G4" s="58"/>
-      <c r="H4" s="58"/>
-      <c r="I4" s="58"/>
-      <c r="J4" s="58"/>
-      <c r="K4" s="58"/>
-      <c r="L4" s="58"/>
-      <c r="M4" s="58"/>
-      <c r="N4" s="58"/>
-      <c r="O4" s="58"/>
-      <c r="P4" s="58"/>
-      <c r="Q4" s="58"/>
-      <c r="R4" s="58"/>
-      <c r="S4" s="58"/>
-      <c r="T4" s="58"/>
-      <c r="U4" s="58"/>
-      <c r="V4" s="58"/>
-      <c r="W4" s="64"/>
-      <c r="X4" s="64"/>
-      <c r="Y4" s="58"/>
-      <c r="Z4" s="58"/>
-      <c r="AA4" s="58"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="47"/>
+      <c r="E4" s="47"/>
+      <c r="F4" s="47"/>
+      <c r="G4" s="47"/>
+      <c r="H4" s="47"/>
+      <c r="I4" s="47"/>
+      <c r="J4" s="47"/>
+      <c r="K4" s="47"/>
+      <c r="L4" s="47"/>
+      <c r="M4" s="47"/>
+      <c r="N4" s="47"/>
+      <c r="O4" s="47"/>
+      <c r="P4" s="47"/>
+      <c r="Q4" s="47"/>
+      <c r="R4" s="47"/>
+      <c r="S4" s="47"/>
+      <c r="T4" s="47"/>
+      <c r="U4" s="47"/>
+      <c r="V4" s="47"/>
+      <c r="W4" s="53"/>
+      <c r="X4" s="53"/>
+      <c r="Y4" s="47"/>
+      <c r="Z4" s="47"/>
+      <c r="AA4" s="47"/>
     </row>
     <row r="5" spans="1:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="58"/>
-      <c r="C5" s="58"/>
-      <c r="D5" s="58"/>
-      <c r="E5" s="58"/>
-      <c r="F5" s="58"/>
-      <c r="G5" s="58"/>
-      <c r="H5" s="58"/>
-      <c r="I5" s="58"/>
-      <c r="J5" s="58"/>
-      <c r="K5" s="58"/>
-      <c r="L5" s="58"/>
-      <c r="M5" s="58"/>
-      <c r="N5" s="58"/>
-      <c r="O5" s="58"/>
-      <c r="P5" s="58"/>
-      <c r="Q5" s="58"/>
-      <c r="R5" s="58"/>
-      <c r="S5" s="58"/>
-      <c r="T5" s="58"/>
-      <c r="U5" s="58"/>
-      <c r="V5" s="58"/>
-      <c r="W5" s="64"/>
-      <c r="X5" s="64"/>
-      <c r="Y5" s="58"/>
-      <c r="Z5" s="58" t="s">
+      <c r="B5" s="47"/>
+      <c r="C5" s="47"/>
+      <c r="D5" s="47"/>
+      <c r="E5" s="47"/>
+      <c r="F5" s="47"/>
+      <c r="G5" s="47"/>
+      <c r="H5" s="47"/>
+      <c r="I5" s="47"/>
+      <c r="J5" s="47"/>
+      <c r="K5" s="47"/>
+      <c r="L5" s="47"/>
+      <c r="M5" s="47"/>
+      <c r="N5" s="47"/>
+      <c r="O5" s="47"/>
+      <c r="P5" s="47"/>
+      <c r="Q5" s="47"/>
+      <c r="R5" s="47"/>
+      <c r="S5" s="47"/>
+      <c r="T5" s="47"/>
+      <c r="U5" s="47"/>
+      <c r="V5" s="47"/>
+      <c r="W5" s="53"/>
+      <c r="X5" s="53"/>
+      <c r="Y5" s="47"/>
+      <c r="Z5" s="47" t="s">
         <v>30</v>
       </c>
-      <c r="AA5" s="58"/>
+      <c r="AA5" s="47"/>
     </row>
     <row r="6" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="58"/>
-      <c r="C6" s="58"/>
-      <c r="D6" s="58"/>
-      <c r="E6" s="58"/>
-      <c r="F6" s="58"/>
-      <c r="G6" s="58"/>
-      <c r="H6" s="58"/>
-      <c r="I6" s="58"/>
-      <c r="J6" s="58"/>
-      <c r="K6" s="58"/>
-      <c r="L6" s="58"/>
-      <c r="M6" s="58"/>
-      <c r="N6" s="58"/>
-      <c r="O6" s="58"/>
-      <c r="P6" s="58"/>
-      <c r="Q6" s="58"/>
-      <c r="R6" s="58"/>
-      <c r="S6" s="58"/>
-      <c r="T6" s="58"/>
-      <c r="U6" s="58"/>
-      <c r="V6" s="58"/>
-      <c r="W6" s="64"/>
-      <c r="X6" s="64"/>
-      <c r="Y6" s="58"/>
-      <c r="Z6" s="58"/>
-      <c r="AA6" s="58"/>
+      <c r="B6" s="47"/>
+      <c r="C6" s="47"/>
+      <c r="D6" s="47"/>
+      <c r="E6" s="47"/>
+      <c r="F6" s="47"/>
+      <c r="G6" s="47"/>
+      <c r="H6" s="47"/>
+      <c r="I6" s="47"/>
+      <c r="J6" s="47"/>
+      <c r="K6" s="47"/>
+      <c r="L6" s="47"/>
+      <c r="M6" s="47"/>
+      <c r="N6" s="47"/>
+      <c r="O6" s="47"/>
+      <c r="P6" s="47"/>
+      <c r="Q6" s="47"/>
+      <c r="R6" s="47"/>
+      <c r="S6" s="47"/>
+      <c r="T6" s="47"/>
+      <c r="U6" s="47"/>
+      <c r="V6" s="47"/>
+      <c r="W6" s="53"/>
+      <c r="X6" s="53"/>
+      <c r="Y6" s="47"/>
+      <c r="Z6" s="47"/>
+      <c r="AA6" s="47"/>
     </row>
     <row r="7" spans="1:27" ht="25.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="60" t="s">
+      <c r="B7" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="61" t="s">
+      <c r="C7" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="61" t="s">
+      <c r="D7" s="50" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="61" t="s">
+      <c r="E7" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="F7" s="61" t="s">
+      <c r="F7" s="50" t="s">
         <v>35</v>
       </c>
-      <c r="G7" s="61" t="s">
+      <c r="G7" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="H7" s="61" t="s">
+      <c r="H7" s="50" t="s">
         <v>37</v>
       </c>
-      <c r="I7" s="61" t="s">
+      <c r="I7" s="50" t="s">
         <v>38</v>
       </c>
-      <c r="J7" s="61" t="s">
+      <c r="J7" s="50" t="s">
         <v>39</v>
       </c>
-      <c r="K7" s="61" t="s">
+      <c r="K7" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="L7" s="61" t="s">
+      <c r="L7" s="50" t="s">
         <v>41</v>
       </c>
-      <c r="M7" s="61" t="s">
+      <c r="M7" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="N7" s="61" t="s">
+      <c r="N7" s="50" t="s">
         <v>42</v>
       </c>
-      <c r="O7" s="61" t="s">
+      <c r="O7" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="P7" s="61" t="s">
+      <c r="P7" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="Q7" s="61" t="s">
+      <c r="Q7" s="50" t="s">
         <v>22</v>
       </c>
-      <c r="R7" s="61" t="s">
+      <c r="R7" s="50" t="s">
         <v>23</v>
       </c>
-      <c r="S7" s="61" t="s">
+      <c r="S7" s="50" t="s">
         <v>43</v>
       </c>
-      <c r="T7" s="61" t="s">
+      <c r="T7" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="U7" s="61" t="s">
+      <c r="U7" s="50" t="s">
         <v>44</v>
       </c>
-      <c r="V7" s="61" t="s">
+      <c r="V7" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="W7" s="63" t="s">
+      <c r="W7" s="52" t="s">
         <v>45</v>
       </c>
-      <c r="X7" s="63" t="s">
+      <c r="X7" s="52" t="s">
         <v>46</v>
       </c>
-      <c r="Y7" s="61" t="s">
+      <c r="Y7" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="Z7" s="61" t="s">
+      <c r="Z7" s="50" t="s">
         <v>228</v>
       </c>
-      <c r="AA7" s="62" t="s">
+      <c r="AA7" s="51" t="s">
         <v>229</v>
       </c>
     </row>
     <row r="8" spans="1:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="53"/>
-      <c r="AA8" s="54"/>
+      <c r="B8" s="42"/>
+      <c r="AA8" s="43"/>
     </row>
     <row r="9" spans="1:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="53"/>
-      <c r="AA9" s="54"/>
+      <c r="B9" s="42"/>
+      <c r="AA9" s="43"/>
     </row>
     <row r="10" spans="1:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="53"/>
-      <c r="AA10" s="54"/>
+      <c r="B10" s="42"/>
+      <c r="AA10" s="43"/>
     </row>
     <row r="11" spans="1:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="53"/>
-      <c r="AA11" s="54"/>
+      <c r="B11" s="42"/>
+      <c r="AA11" s="43"/>
     </row>
     <row r="12" spans="1:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="53"/>
-      <c r="AA12" s="54"/>
+      <c r="B12" s="42"/>
+      <c r="AA12" s="43"/>
     </row>
     <row r="13" spans="1:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="53"/>
-      <c r="AA13" s="54"/>
+      <c r="B13" s="42"/>
+      <c r="AA13" s="43"/>
     </row>
     <row r="14" spans="1:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="53"/>
-      <c r="AA14" s="54"/>
+      <c r="B14" s="42"/>
+      <c r="AA14" s="43"/>
     </row>
     <row r="15" spans="1:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="53"/>
-      <c r="AA15" s="54"/>
+      <c r="B15" s="42"/>
+      <c r="AA15" s="43"/>
     </row>
     <row r="16" spans="1:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="53"/>
-      <c r="AA16" s="54"/>
+      <c r="B16" s="42"/>
+      <c r="AA16" s="43"/>
     </row>
     <row r="17" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="53"/>
-      <c r="AA17" s="54"/>
+      <c r="B17" s="42"/>
+      <c r="AA17" s="43"/>
     </row>
     <row r="18" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="53"/>
-      <c r="AA18" s="54"/>
+      <c r="B18" s="42"/>
+      <c r="AA18" s="43"/>
     </row>
     <row r="19" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="53"/>
-      <c r="AA19" s="54"/>
+      <c r="B19" s="42"/>
+      <c r="AA19" s="43"/>
     </row>
     <row r="20" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="53"/>
-      <c r="AA20" s="54"/>
+      <c r="B20" s="42"/>
+      <c r="AA20" s="43"/>
     </row>
     <row r="21" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="53"/>
-      <c r="AA21" s="54"/>
+      <c r="B21" s="42"/>
+      <c r="AA21" s="43"/>
     </row>
     <row r="22" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="53"/>
-      <c r="AA22" s="54"/>
+      <c r="B22" s="42"/>
+      <c r="AA22" s="43"/>
     </row>
     <row r="23" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="53"/>
-      <c r="AA23" s="54"/>
+      <c r="B23" s="42"/>
+      <c r="AA23" s="43"/>
     </row>
     <row r="24" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="53"/>
-      <c r="AA24" s="54"/>
+      <c r="B24" s="42"/>
+      <c r="AA24" s="43"/>
     </row>
     <row r="25" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="53"/>
-      <c r="AA25" s="54"/>
+      <c r="B25" s="42"/>
+      <c r="AA25" s="43"/>
     </row>
     <row r="26" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="53"/>
-      <c r="AA26" s="54"/>
+      <c r="B26" s="42"/>
+      <c r="AA26" s="43"/>
     </row>
     <row r="27" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="53"/>
-      <c r="AA27" s="54"/>
+      <c r="B27" s="42"/>
+      <c r="AA27" s="43"/>
     </row>
     <row r="28" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="53"/>
-      <c r="AA28" s="54"/>
+      <c r="B28" s="42"/>
+      <c r="AA28" s="43"/>
     </row>
     <row r="29" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="53"/>
-      <c r="AA29" s="54"/>
+      <c r="B29" s="42"/>
+      <c r="AA29" s="43"/>
     </row>
     <row r="30" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="53"/>
-      <c r="AA30" s="54"/>
+      <c r="B30" s="42"/>
+      <c r="AA30" s="43"/>
     </row>
     <row r="31" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="53"/>
-      <c r="AA31" s="54"/>
+      <c r="B31" s="42"/>
+      <c r="AA31" s="43"/>
     </row>
     <row r="32" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="53"/>
-      <c r="AA32" s="54"/>
+      <c r="B32" s="42"/>
+      <c r="AA32" s="43"/>
     </row>
     <row r="33" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="53"/>
-      <c r="AA33" s="54"/>
+      <c r="B33" s="42"/>
+      <c r="AA33" s="43"/>
     </row>
     <row r="34" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="53"/>
-      <c r="AA34" s="54"/>
+      <c r="B34" s="42"/>
+      <c r="AA34" s="43"/>
     </row>
     <row r="35" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="53"/>
-      <c r="AA35" s="54"/>
+      <c r="B35" s="42"/>
+      <c r="AA35" s="43"/>
     </row>
     <row r="36" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="53"/>
-      <c r="AA36" s="54"/>
+      <c r="B36" s="42"/>
+      <c r="AA36" s="43"/>
     </row>
     <row r="37" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="53"/>
-      <c r="AA37" s="54"/>
+      <c r="B37" s="42"/>
+      <c r="AA37" s="43"/>
     </row>
     <row r="38" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="53"/>
-      <c r="AA38" s="54"/>
+      <c r="B38" s="42"/>
+      <c r="AA38" s="43"/>
     </row>
     <row r="39" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="53"/>
-      <c r="AA39" s="54"/>
+      <c r="B39" s="42"/>
+      <c r="AA39" s="43"/>
     </row>
     <row r="40" spans="2:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="53"/>
-      <c r="AA40" s="54"/>
+      <c r="B40" s="42"/>
+      <c r="AA40" s="43"/>
     </row>
     <row r="41" spans="2:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="53"/>
-      <c r="AA41" s="54"/>
+      <c r="B41" s="42"/>
+      <c r="AA41" s="43"/>
     </row>
     <row r="42" spans="2:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="53"/>
-      <c r="AA42" s="54"/>
+      <c r="B42" s="42"/>
+      <c r="AA42" s="43"/>
     </row>
     <row r="43" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="53"/>
-      <c r="AA43" s="54"/>
+      <c r="B43" s="42"/>
+      <c r="AA43" s="43"/>
     </row>
     <row r="44" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="53"/>
-      <c r="AA44" s="54"/>
+      <c r="B44" s="42"/>
+      <c r="AA44" s="43"/>
     </row>
     <row r="45" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="53"/>
-      <c r="AA45" s="54"/>
+      <c r="B45" s="42"/>
+      <c r="AA45" s="43"/>
     </row>
     <row r="46" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="53"/>
-      <c r="AA46" s="54"/>
+      <c r="B46" s="42"/>
+      <c r="AA46" s="43"/>
     </row>
     <row r="47" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="53"/>
-      <c r="AA47" s="54"/>
+      <c r="B47" s="42"/>
+      <c r="AA47" s="43"/>
     </row>
     <row r="48" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="53"/>
-      <c r="AA48" s="54"/>
+      <c r="B48" s="42"/>
+      <c r="AA48" s="43"/>
     </row>
     <row r="49" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="53"/>
-      <c r="AA49" s="54"/>
+      <c r="B49" s="42"/>
+      <c r="AA49" s="43"/>
     </row>
     <row r="50" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="53"/>
-      <c r="AA50" s="54"/>
+      <c r="B50" s="42"/>
+      <c r="AA50" s="43"/>
     </row>
     <row r="51" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="53"/>
-      <c r="AA51" s="54"/>
+      <c r="B51" s="42"/>
+      <c r="AA51" s="43"/>
     </row>
     <row r="52" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="53"/>
-      <c r="AA52" s="54"/>
+      <c r="B52" s="42"/>
+      <c r="AA52" s="43"/>
     </row>
     <row r="53" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="53"/>
-      <c r="AA53" s="54"/>
+      <c r="B53" s="42"/>
+      <c r="AA53" s="43"/>
     </row>
     <row r="54" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="53"/>
-      <c r="AA54" s="54"/>
+      <c r="B54" s="42"/>
+      <c r="AA54" s="43"/>
     </row>
     <row r="55" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="53"/>
-      <c r="AA55" s="54"/>
+      <c r="B55" s="42"/>
+      <c r="AA55" s="43"/>
     </row>
     <row r="56" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B56" s="53"/>
-      <c r="AA56" s="54"/>
+      <c r="B56" s="42"/>
+      <c r="AA56" s="43"/>
     </row>
     <row r="57" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="53"/>
-      <c r="AA57" s="54"/>
+      <c r="B57" s="42"/>
+      <c r="AA57" s="43"/>
     </row>
     <row r="58" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="53"/>
-      <c r="AA58" s="54"/>
+      <c r="B58" s="42"/>
+      <c r="AA58" s="43"/>
     </row>
     <row r="59" spans="2:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="53"/>
-      <c r="AA59" s="54"/>
+      <c r="B59" s="42"/>
+      <c r="AA59" s="43"/>
     </row>
     <row r="60" spans="2:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="53"/>
-      <c r="AA60" s="54"/>
+      <c r="B60" s="42"/>
+      <c r="AA60" s="43"/>
     </row>
     <row r="61" spans="2:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="53"/>
-      <c r="AA61" s="54"/>
+      <c r="B61" s="42"/>
+      <c r="AA61" s="43"/>
     </row>
     <row r="62" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="53"/>
-      <c r="AA62" s="54"/>
+      <c r="B62" s="42"/>
+      <c r="AA62" s="43"/>
     </row>
     <row r="63" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="53"/>
-      <c r="AA63" s="54"/>
+      <c r="B63" s="42"/>
+      <c r="AA63" s="43"/>
     </row>
     <row r="64" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B64" s="53"/>
-      <c r="AA64" s="54"/>
+      <c r="B64" s="42"/>
+      <c r="AA64" s="43"/>
     </row>
     <row r="65" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="53"/>
-      <c r="AA65" s="54"/>
+      <c r="B65" s="42"/>
+      <c r="AA65" s="43"/>
     </row>
     <row r="66" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="53"/>
-      <c r="AA66" s="54"/>
+      <c r="B66" s="42"/>
+      <c r="AA66" s="43"/>
     </row>
     <row r="67" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="53"/>
-      <c r="AA67" s="54"/>
+      <c r="B67" s="42"/>
+      <c r="AA67" s="43"/>
     </row>
     <row r="68" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B68" s="53"/>
-      <c r="AA68" s="54"/>
+      <c r="B68" s="42"/>
+      <c r="AA68" s="43"/>
     </row>
     <row r="69" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B69" s="53"/>
-      <c r="AA69" s="54"/>
+      <c r="B69" s="42"/>
+      <c r="AA69" s="43"/>
     </row>
     <row r="70" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B70" s="53"/>
-      <c r="AA70" s="54"/>
+      <c r="B70" s="42"/>
+      <c r="AA70" s="43"/>
     </row>
     <row r="71" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B71" s="53"/>
-      <c r="AA71" s="54"/>
+      <c r="B71" s="42"/>
+      <c r="AA71" s="43"/>
     </row>
     <row r="72" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B72" s="53"/>
-      <c r="AA72" s="54"/>
+      <c r="B72" s="42"/>
+      <c r="AA72" s="43"/>
     </row>
     <row r="73" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B73" s="53"/>
-      <c r="AA73" s="54"/>
+      <c r="B73" s="42"/>
+      <c r="AA73" s="43"/>
     </row>
     <row r="74" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B74" s="53"/>
-      <c r="AA74" s="54"/>
+      <c r="B74" s="42"/>
+      <c r="AA74" s="43"/>
     </row>
     <row r="75" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B75" s="53"/>
-      <c r="AA75" s="54"/>
+      <c r="B75" s="42"/>
+      <c r="AA75" s="43"/>
     </row>
     <row r="76" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B76" s="53"/>
-      <c r="AA76" s="54"/>
+      <c r="B76" s="42"/>
+      <c r="AA76" s="43"/>
     </row>
     <row r="77" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B77" s="53"/>
-      <c r="AA77" s="54"/>
+      <c r="B77" s="42"/>
+      <c r="AA77" s="43"/>
     </row>
     <row r="78" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B78" s="53"/>
-      <c r="AA78" s="54"/>
+      <c r="B78" s="42"/>
+      <c r="AA78" s="43"/>
     </row>
     <row r="79" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B79" s="53"/>
-      <c r="AA79" s="54"/>
+      <c r="B79" s="42"/>
+      <c r="AA79" s="43"/>
     </row>
     <row r="80" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B80" s="53"/>
-      <c r="AA80" s="54"/>
+      <c r="B80" s="42"/>
+      <c r="AA80" s="43"/>
     </row>
     <row r="81" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B81" s="53"/>
-      <c r="AA81" s="54"/>
+      <c r="B81" s="42"/>
+      <c r="AA81" s="43"/>
     </row>
     <row r="82" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B82" s="53"/>
-      <c r="AA82" s="54"/>
+      <c r="B82" s="42"/>
+      <c r="AA82" s="43"/>
     </row>
     <row r="83" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B83" s="53"/>
-      <c r="AA83" s="54"/>
+      <c r="B83" s="42"/>
+      <c r="AA83" s="43"/>
     </row>
     <row r="84" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B84" s="53"/>
-      <c r="AA84" s="54"/>
+      <c r="B84" s="42"/>
+      <c r="AA84" s="43"/>
     </row>
     <row r="85" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B85" s="53"/>
-      <c r="AA85" s="54"/>
+      <c r="B85" s="42"/>
+      <c r="AA85" s="43"/>
     </row>
     <row r="86" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B86" s="53"/>
-      <c r="AA86" s="54"/>
+      <c r="B86" s="42"/>
+      <c r="AA86" s="43"/>
     </row>
     <row r="87" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B87" s="53"/>
-      <c r="AA87" s="54"/>
+      <c r="B87" s="42"/>
+      <c r="AA87" s="43"/>
     </row>
     <row r="88" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B88" s="53"/>
-      <c r="AA88" s="54"/>
+      <c r="B88" s="42"/>
+      <c r="AA88" s="43"/>
     </row>
     <row r="89" spans="2:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B89" s="53"/>
-      <c r="AA89" s="54"/>
+      <c r="B89" s="42"/>
+      <c r="AA89" s="43"/>
     </row>
     <row r="90" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B90" s="53"/>
-      <c r="AA90" s="54"/>
+      <c r="B90" s="42"/>
+      <c r="AA90" s="43"/>
     </row>
     <row r="91" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B91" s="53"/>
-      <c r="AA91" s="54"/>
+      <c r="B91" s="42"/>
+      <c r="AA91" s="43"/>
     </row>
     <row r="92" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B92" s="53"/>
-      <c r="AA92" s="54"/>
+      <c r="B92" s="42"/>
+      <c r="AA92" s="43"/>
     </row>
     <row r="93" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B93" s="53"/>
-      <c r="AA93" s="54"/>
+      <c r="B93" s="42"/>
+      <c r="AA93" s="43"/>
     </row>
     <row r="94" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B94" s="53"/>
-      <c r="AA94" s="54"/>
+      <c r="B94" s="42"/>
+      <c r="AA94" s="43"/>
     </row>
     <row r="95" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B95" s="53"/>
-      <c r="AA95" s="54"/>
+      <c r="B95" s="42"/>
+      <c r="AA95" s="43"/>
     </row>
     <row r="96" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B96" s="53"/>
-      <c r="AA96" s="54"/>
+      <c r="B96" s="42"/>
+      <c r="AA96" s="43"/>
     </row>
     <row r="97" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B97" s="53"/>
-      <c r="AA97" s="54"/>
+      <c r="B97" s="42"/>
+      <c r="AA97" s="43"/>
     </row>
     <row r="98" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B98" s="53"/>
-      <c r="AA98" s="54"/>
+      <c r="B98" s="42"/>
+      <c r="AA98" s="43"/>
     </row>
     <row r="99" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B99" s="53"/>
-      <c r="AA99" s="54"/>
+      <c r="B99" s="42"/>
+      <c r="AA99" s="43"/>
     </row>
     <row r="100" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B100" s="53"/>
-      <c r="AA100" s="54"/>
+      <c r="B100" s="42"/>
+      <c r="AA100" s="43"/>
     </row>
     <row r="101" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B101" s="53"/>
-      <c r="AA101" s="54"/>
+      <c r="B101" s="42"/>
+      <c r="AA101" s="43"/>
     </row>
     <row r="102" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B102" s="53"/>
-      <c r="AA102" s="54"/>
+      <c r="B102" s="42"/>
+      <c r="AA102" s="43"/>
     </row>
     <row r="103" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B103" s="53"/>
-      <c r="AA103" s="54"/>
+      <c r="B103" s="42"/>
+      <c r="AA103" s="43"/>
     </row>
     <row r="104" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B104" s="53"/>
-      <c r="AA104" s="54"/>
+      <c r="B104" s="42"/>
+      <c r="AA104" s="43"/>
     </row>
     <row r="105" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B105" s="53"/>
-      <c r="AA105" s="54"/>
+      <c r="B105" s="42"/>
+      <c r="AA105" s="43"/>
     </row>
     <row r="106" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B106" s="53"/>
-      <c r="AA106" s="54"/>
+      <c r="B106" s="42"/>
+      <c r="AA106" s="43"/>
     </row>
     <row r="107" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B107" s="53"/>
-      <c r="AA107" s="54"/>
+      <c r="B107" s="42"/>
+      <c r="AA107" s="43"/>
     </row>
     <row r="108" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B108" s="53"/>
-      <c r="AA108" s="54"/>
+      <c r="B108" s="42"/>
+      <c r="AA108" s="43"/>
     </row>
     <row r="109" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B109" s="53"/>
-      <c r="AA109" s="54"/>
+      <c r="B109" s="42"/>
+      <c r="AA109" s="43"/>
     </row>
     <row r="110" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B110" s="53"/>
-      <c r="AA110" s="54"/>
+      <c r="B110" s="42"/>
+      <c r="AA110" s="43"/>
     </row>
     <row r="111" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B111" s="53"/>
-      <c r="AA111" s="54"/>
+      <c r="B111" s="42"/>
+      <c r="AA111" s="43"/>
     </row>
     <row r="112" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B112" s="53"/>
-      <c r="AA112" s="54"/>
+      <c r="B112" s="42"/>
+      <c r="AA112" s="43"/>
     </row>
     <row r="113" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B113" s="53"/>
-      <c r="AA113" s="54"/>
+      <c r="B113" s="42"/>
+      <c r="AA113" s="43"/>
     </row>
     <row r="114" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B114" s="53"/>
-      <c r="AA114" s="54"/>
+      <c r="B114" s="42"/>
+      <c r="AA114" s="43"/>
     </row>
     <row r="115" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B115" s="53"/>
-      <c r="AA115" s="54"/>
+      <c r="B115" s="42"/>
+      <c r="AA115" s="43"/>
     </row>
     <row r="116" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B116" s="53"/>
-      <c r="AA116" s="54"/>
+      <c r="B116" s="42"/>
+      <c r="AA116" s="43"/>
     </row>
     <row r="117" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B117" s="53"/>
-      <c r="AA117" s="54"/>
+      <c r="B117" s="42"/>
+      <c r="AA117" s="43"/>
     </row>
     <row r="118" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B118" s="53"/>
-      <c r="AA118" s="54"/>
+      <c r="B118" s="42"/>
+      <c r="AA118" s="43"/>
     </row>
     <row r="119" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B119" s="53"/>
-      <c r="AA119" s="54"/>
+      <c r="B119" s="42"/>
+      <c r="AA119" s="43"/>
     </row>
     <row r="120" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B120" s="53"/>
-      <c r="AA120" s="54"/>
+      <c r="B120" s="42"/>
+      <c r="AA120" s="43"/>
     </row>
     <row r="121" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B121" s="53"/>
-      <c r="AA121" s="54"/>
+      <c r="B121" s="42"/>
+      <c r="AA121" s="43"/>
     </row>
     <row r="122" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B122" s="53"/>
-      <c r="AA122" s="54"/>
+      <c r="B122" s="42"/>
+      <c r="AA122" s="43"/>
     </row>
     <row r="123" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B123" s="53"/>
-      <c r="AA123" s="54"/>
+      <c r="B123" s="42"/>
+      <c r="AA123" s="43"/>
     </row>
     <row r="124" spans="2:27" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B124" s="53"/>
-      <c r="AA124" s="54"/>
+      <c r="B124" s="42"/>
+      <c r="AA124" s="43"/>
     </row>
     <row r="125" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B125" s="53"/>
-      <c r="AA125" s="54"/>
+      <c r="B125" s="42"/>
+      <c r="AA125" s="43"/>
     </row>
     <row r="126" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B126" s="53"/>
-      <c r="AA126" s="54"/>
+      <c r="B126" s="42"/>
+      <c r="AA126" s="43"/>
     </row>
     <row r="127" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B127" s="53"/>
-      <c r="AA127" s="54"/>
+      <c r="B127" s="42"/>
+      <c r="AA127" s="43"/>
     </row>
     <row r="128" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B128" s="53"/>
-      <c r="AA128" s="54"/>
+      <c r="B128" s="42"/>
+      <c r="AA128" s="43"/>
     </row>
     <row r="129" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B129" s="53"/>
-      <c r="AA129" s="54"/>
+      <c r="B129" s="42"/>
+      <c r="AA129" s="43"/>
     </row>
     <row r="130" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B130" s="53"/>
-      <c r="AA130" s="54"/>
+      <c r="B130" s="42"/>
+      <c r="AA130" s="43"/>
     </row>
     <row r="131" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B131" s="53"/>
-      <c r="AA131" s="54"/>
+      <c r="B131" s="42"/>
+      <c r="AA131" s="43"/>
     </row>
     <row r="132" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B132" s="53"/>
-      <c r="AA132" s="54"/>
+      <c r="B132" s="42"/>
+      <c r="AA132" s="43"/>
     </row>
     <row r="133" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B133" s="53"/>
-      <c r="AA133" s="54"/>
+      <c r="B133" s="42"/>
+      <c r="AA133" s="43"/>
     </row>
     <row r="134" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B134" s="53"/>
-      <c r="AA134" s="54"/>
+      <c r="B134" s="42"/>
+      <c r="AA134" s="43"/>
     </row>
     <row r="135" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B135" s="53"/>
-      <c r="AA135" s="54"/>
+      <c r="B135" s="42"/>
+      <c r="AA135" s="43"/>
     </row>
     <row r="136" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B136" s="53"/>
-      <c r="AA136" s="54"/>
+      <c r="B136" s="42"/>
+      <c r="AA136" s="43"/>
     </row>
     <row r="137" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B137" s="53"/>
-      <c r="AA137" s="54"/>
+      <c r="B137" s="42"/>
+      <c r="AA137" s="43"/>
     </row>
     <row r="138" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B138" s="53"/>
-      <c r="AA138" s="54"/>
+      <c r="B138" s="42"/>
+      <c r="AA138" s="43"/>
     </row>
     <row r="139" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B139" s="53"/>
-      <c r="AA139" s="54"/>
+      <c r="B139" s="42"/>
+      <c r="AA139" s="43"/>
     </row>
     <row r="140" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B140" s="53"/>
-      <c r="AA140" s="54"/>
+      <c r="B140" s="42"/>
+      <c r="AA140" s="43"/>
     </row>
     <row r="141" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B141" s="53"/>
-      <c r="AA141" s="54"/>
+      <c r="B141" s="42"/>
+      <c r="AA141" s="43"/>
     </row>
     <row r="142" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B142" s="53"/>
-      <c r="AA142" s="54"/>
+      <c r="B142" s="42"/>
+      <c r="AA142" s="43"/>
     </row>
     <row r="143" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B143" s="53"/>
-      <c r="AA143" s="54"/>
+      <c r="B143" s="42"/>
+      <c r="AA143" s="43"/>
     </row>
     <row r="144" spans="2:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B144" s="53"/>
-      <c r="AA144" s="54"/>
+      <c r="B144" s="42"/>
+      <c r="AA144" s="43"/>
     </row>
     <row r="145" spans="2:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B145" s="53"/>
-      <c r="AA145" s="54"/>
+      <c r="B145" s="42"/>
+      <c r="AA145" s="43"/>
     </row>
     <row r="146" spans="2:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B146" s="53"/>
-      <c r="AA146" s="54"/>
+      <c r="B146" s="42"/>
+      <c r="AA146" s="43"/>
     </row>
     <row r="147" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B147" s="53"/>
-      <c r="AA147" s="54"/>
+      <c r="B147" s="42"/>
+      <c r="AA147" s="43"/>
     </row>
     <row r="148" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B148" s="53"/>
-      <c r="AA148" s="54"/>
+      <c r="B148" s="42"/>
+      <c r="AA148" s="43"/>
     </row>
     <row r="149" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B149" s="53"/>
-      <c r="AA149" s="54"/>
+      <c r="B149" s="42"/>
+      <c r="AA149" s="43"/>
     </row>
     <row r="150" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B150" s="53"/>
-      <c r="AA150" s="54"/>
+      <c r="B150" s="42"/>
+      <c r="AA150" s="43"/>
     </row>
     <row r="151" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B151" s="53"/>
-      <c r="AA151" s="54"/>
+      <c r="B151" s="42"/>
+      <c r="AA151" s="43"/>
     </row>
     <row r="152" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B152" s="53"/>
-      <c r="AA152" s="54"/>
+      <c r="B152" s="42"/>
+      <c r="AA152" s="43"/>
     </row>
     <row r="153" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B153" s="53"/>
-      <c r="AA153" s="54"/>
+      <c r="B153" s="42"/>
+      <c r="AA153" s="43"/>
     </row>
     <row r="154" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B154" s="53"/>
-      <c r="AA154" s="54"/>
+      <c r="B154" s="42"/>
+      <c r="AA154" s="43"/>
     </row>
     <row r="155" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B155" s="53"/>
-      <c r="AA155" s="54"/>
+      <c r="B155" s="42"/>
+      <c r="AA155" s="43"/>
     </row>
     <row r="156" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B156" s="53"/>
-      <c r="AA156" s="54"/>
+      <c r="B156" s="42"/>
+      <c r="AA156" s="43"/>
     </row>
     <row r="157" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B157" s="53"/>
-      <c r="AA157" s="54"/>
+      <c r="B157" s="42"/>
+      <c r="AA157" s="43"/>
     </row>
     <row r="158" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B158" s="53"/>
-      <c r="AA158" s="54"/>
+      <c r="B158" s="42"/>
+      <c r="AA158" s="43"/>
     </row>
     <row r="159" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B159" s="53"/>
-      <c r="AA159" s="54"/>
+      <c r="B159" s="42"/>
+      <c r="AA159" s="43"/>
     </row>
     <row r="160" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B160" s="53"/>
-      <c r="AA160" s="54"/>
+      <c r="B160" s="42"/>
+      <c r="AA160" s="43"/>
     </row>
     <row r="161" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B161" s="53"/>
-      <c r="AA161" s="54"/>
+      <c r="B161" s="42"/>
+      <c r="AA161" s="43"/>
     </row>
     <row r="162" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B162" s="53"/>
-      <c r="AA162" s="54"/>
+      <c r="B162" s="42"/>
+      <c r="AA162" s="43"/>
     </row>
     <row r="163" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B163" s="53"/>
-      <c r="AA163" s="54"/>
+      <c r="B163" s="42"/>
+      <c r="AA163" s="43"/>
     </row>
     <row r="164" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B164" s="53"/>
-      <c r="AA164" s="54"/>
+      <c r="B164" s="42"/>
+      <c r="AA164" s="43"/>
     </row>
     <row r="165" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B165" s="53"/>
-      <c r="AA165" s="54"/>
+      <c r="B165" s="42"/>
+      <c r="AA165" s="43"/>
     </row>
     <row r="166" spans="2:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B166" s="53"/>
-      <c r="AA166" s="54"/>
+      <c r="B166" s="42"/>
+      <c r="AA166" s="43"/>
     </row>
     <row r="167" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B167" s="53"/>
-      <c r="AA167" s="54"/>
+      <c r="B167" s="42"/>
+      <c r="AA167" s="43"/>
     </row>
     <row r="168" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B168" s="53"/>
-      <c r="AA168" s="54"/>
+      <c r="B168" s="42"/>
+      <c r="AA168" s="43"/>
     </row>
     <row r="169" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B169" s="53"/>
-      <c r="AA169" s="54"/>
+      <c r="B169" s="42"/>
+      <c r="AA169" s="43"/>
     </row>
     <row r="170" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B170" s="53"/>
-      <c r="AA170" s="54"/>
+      <c r="B170" s="42"/>
+      <c r="AA170" s="43"/>
     </row>
     <row r="171" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B171" s="53"/>
-      <c r="AA171" s="54"/>
+      <c r="B171" s="42"/>
+      <c r="AA171" s="43"/>
     </row>
     <row r="172" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B172" s="53"/>
-      <c r="AA172" s="54"/>
+      <c r="B172" s="42"/>
+      <c r="AA172" s="43"/>
     </row>
     <row r="173" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B173" s="53"/>
-      <c r="AA173" s="54"/>
+      <c r="B173" s="42"/>
+      <c r="AA173" s="43"/>
     </row>
     <row r="174" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B174" s="53"/>
-      <c r="AA174" s="54"/>
+      <c r="B174" s="42"/>
+      <c r="AA174" s="43"/>
     </row>
     <row r="175" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B175" s="53"/>
-      <c r="AA175" s="54"/>
+      <c r="B175" s="42"/>
+      <c r="AA175" s="43"/>
     </row>
     <row r="176" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B176" s="53"/>
-      <c r="AA176" s="54"/>
+      <c r="B176" s="42"/>
+      <c r="AA176" s="43"/>
     </row>
     <row r="177" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B177" s="53"/>
-      <c r="AA177" s="54"/>
+      <c r="B177" s="42"/>
+      <c r="AA177" s="43"/>
     </row>
     <row r="178" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B178" s="53"/>
-      <c r="AA178" s="54"/>
+      <c r="B178" s="42"/>
+      <c r="AA178" s="43"/>
     </row>
     <row r="179" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B179" s="53"/>
-      <c r="AA179" s="54"/>
+      <c r="B179" s="42"/>
+      <c r="AA179" s="43"/>
     </row>
     <row r="180" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B180" s="53"/>
-      <c r="AA180" s="54"/>
+      <c r="B180" s="42"/>
+      <c r="AA180" s="43"/>
     </row>
     <row r="181" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B181" s="53"/>
-      <c r="AA181" s="54"/>
+      <c r="B181" s="42"/>
+      <c r="AA181" s="43"/>
     </row>
     <row r="182" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B182" s="53"/>
-      <c r="AA182" s="54"/>
+      <c r="B182" s="42"/>
+      <c r="AA182" s="43"/>
     </row>
     <row r="183" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B183" s="53"/>
-      <c r="AA183" s="54"/>
+      <c r="B183" s="42"/>
+      <c r="AA183" s="43"/>
     </row>
     <row r="184" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B184" s="53"/>
-      <c r="AA184" s="54"/>
+      <c r="B184" s="42"/>
+      <c r="AA184" s="43"/>
     </row>
     <row r="185" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B185" s="53"/>
-      <c r="AA185" s="54"/>
+      <c r="B185" s="42"/>
+      <c r="AA185" s="43"/>
     </row>
     <row r="186" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B186" s="53"/>
-      <c r="AA186" s="54"/>
+      <c r="B186" s="42"/>
+      <c r="AA186" s="43"/>
     </row>
     <row r="187" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B187" s="53"/>
-      <c r="AA187" s="54"/>
+      <c r="B187" s="42"/>
+      <c r="AA187" s="43"/>
     </row>
     <row r="188" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B188" s="53"/>
-      <c r="AA188" s="54"/>
+      <c r="B188" s="42"/>
+      <c r="AA188" s="43"/>
     </row>
     <row r="189" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B189" s="53"/>
-      <c r="AA189" s="54"/>
+      <c r="B189" s="42"/>
+      <c r="AA189" s="43"/>
     </row>
     <row r="190" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B190" s="53"/>
-      <c r="AA190" s="54"/>
+      <c r="B190" s="42"/>
+      <c r="AA190" s="43"/>
     </row>
     <row r="191" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B191" s="53"/>
-      <c r="AA191" s="54"/>
+      <c r="B191" s="42"/>
+      <c r="AA191" s="43"/>
     </row>
     <row r="192" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B192" s="53"/>
-      <c r="AA192" s="54"/>
+      <c r="B192" s="42"/>
+      <c r="AA192" s="43"/>
     </row>
     <row r="193" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B193" s="53"/>
-      <c r="AA193" s="54"/>
+      <c r="B193" s="42"/>
+      <c r="AA193" s="43"/>
     </row>
     <row r="194" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B194" s="53"/>
-      <c r="AA194" s="54"/>
+      <c r="B194" s="42"/>
+      <c r="AA194" s="43"/>
     </row>
     <row r="195" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B195" s="53"/>
-      <c r="AA195" s="54"/>
+      <c r="B195" s="42"/>
+      <c r="AA195" s="43"/>
     </row>
     <row r="196" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B196" s="53"/>
-      <c r="AA196" s="54"/>
+      <c r="B196" s="42"/>
+      <c r="AA196" s="43"/>
     </row>
     <row r="197" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B197" s="53"/>
-      <c r="AA197" s="54"/>
+      <c r="B197" s="42"/>
+      <c r="AA197" s="43"/>
     </row>
     <row r="198" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B198" s="53"/>
-      <c r="AA198" s="54"/>
+      <c r="B198" s="42"/>
+      <c r="AA198" s="43"/>
     </row>
     <row r="199" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B199" s="53"/>
-      <c r="AA199" s="54"/>
+      <c r="B199" s="42"/>
+      <c r="AA199" s="43"/>
     </row>
     <row r="200" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B200" s="53"/>
-      <c r="AA200" s="54"/>
+      <c r="B200" s="42"/>
+      <c r="AA200" s="43"/>
     </row>
     <row r="201" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B201" s="53"/>
-      <c r="AA201" s="54"/>
+      <c r="B201" s="42"/>
+      <c r="AA201" s="43"/>
     </row>
     <row r="202" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B202" s="53"/>
-      <c r="AA202" s="54"/>
+      <c r="B202" s="42"/>
+      <c r="AA202" s="43"/>
     </row>
     <row r="203" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B203" s="53"/>
-      <c r="AA203" s="54"/>
+      <c r="B203" s="42"/>
+      <c r="AA203" s="43"/>
     </row>
     <row r="204" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B204" s="53"/>
-      <c r="AA204" s="54"/>
+      <c r="B204" s="42"/>
+      <c r="AA204" s="43"/>
     </row>
     <row r="205" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B205" s="53"/>
-      <c r="AA205" s="54"/>
+      <c r="B205" s="42"/>
+      <c r="AA205" s="43"/>
     </row>
     <row r="206" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B206" s="53"/>
-      <c r="AA206" s="54"/>
+      <c r="B206" s="42"/>
+      <c r="AA206" s="43"/>
     </row>
     <row r="207" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B207" s="53"/>
-      <c r="AA207" s="54"/>
+      <c r="B207" s="42"/>
+      <c r="AA207" s="43"/>
     </row>
     <row r="208" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B208" s="53"/>
-      <c r="AA208" s="54"/>
+      <c r="B208" s="42"/>
+      <c r="AA208" s="43"/>
     </row>
     <row r="209" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B209" s="53"/>
-      <c r="AA209" s="54"/>
+      <c r="B209" s="42"/>
+      <c r="AA209" s="43"/>
     </row>
     <row r="210" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B210" s="53"/>
-      <c r="AA210" s="54"/>
+      <c r="B210" s="42"/>
+      <c r="AA210" s="43"/>
     </row>
     <row r="211" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B211" s="53"/>
-      <c r="AA211" s="54"/>
+      <c r="B211" s="42"/>
+      <c r="AA211" s="43"/>
     </row>
     <row r="212" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B212" s="53"/>
-      <c r="AA212" s="54"/>
+      <c r="B212" s="42"/>
+      <c r="AA212" s="43"/>
     </row>
     <row r="213" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B213" s="53"/>
-      <c r="AA213" s="54"/>
+      <c r="B213" s="42"/>
+      <c r="AA213" s="43"/>
     </row>
     <row r="214" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B214" s="53"/>
-      <c r="AA214" s="54"/>
+      <c r="B214" s="42"/>
+      <c r="AA214" s="43"/>
     </row>
     <row r="215" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B215" s="53"/>
-      <c r="AA215" s="54"/>
+      <c r="B215" s="42"/>
+      <c r="AA215" s="43"/>
     </row>
     <row r="216" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B216" s="53"/>
-      <c r="AA216" s="54"/>
+      <c r="B216" s="42"/>
+      <c r="AA216" s="43"/>
     </row>
     <row r="217" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B217" s="53"/>
-      <c r="AA217" s="54"/>
+      <c r="B217" s="42"/>
+      <c r="AA217" s="43"/>
     </row>
     <row r="218" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B218" s="53"/>
-      <c r="AA218" s="54"/>
+      <c r="B218" s="42"/>
+      <c r="AA218" s="43"/>
     </row>
     <row r="219" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B219" s="53"/>
-      <c r="AA219" s="54"/>
+      <c r="B219" s="42"/>
+      <c r="AA219" s="43"/>
     </row>
     <row r="220" spans="2:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B220" s="53"/>
-      <c r="AA220" s="54"/>
+      <c r="B220" s="42"/>
+      <c r="AA220" s="43"/>
     </row>
     <row r="221" spans="2:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B221" s="53"/>
-      <c r="AA221" s="54"/>
+      <c r="B221" s="42"/>
+      <c r="AA221" s="43"/>
     </row>
     <row r="222" spans="2:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B222" s="53"/>
-      <c r="AA222" s="54"/>
+      <c r="B222" s="42"/>
+      <c r="AA222" s="43"/>
     </row>
     <row r="223" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B223" s="53"/>
-      <c r="AA223" s="54"/>
+      <c r="B223" s="42"/>
+      <c r="AA223" s="43"/>
     </row>
     <row r="224" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B224" s="53"/>
-      <c r="AA224" s="54"/>
+      <c r="B224" s="42"/>
+      <c r="AA224" s="43"/>
     </row>
     <row r="225" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B225" s="53"/>
-      <c r="AA225" s="54"/>
+      <c r="B225" s="42"/>
+      <c r="AA225" s="43"/>
     </row>
     <row r="226" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B226" s="53"/>
-      <c r="AA226" s="54"/>
+      <c r="B226" s="42"/>
+      <c r="AA226" s="43"/>
     </row>
     <row r="227" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B227" s="53"/>
-      <c r="AA227" s="54"/>
+      <c r="B227" s="42"/>
+      <c r="AA227" s="43"/>
     </row>
     <row r="228" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B228" s="53"/>
-      <c r="AA228" s="54"/>
+      <c r="B228" s="42"/>
+      <c r="AA228" s="43"/>
     </row>
     <row r="229" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B229" s="53"/>
-      <c r="AA229" s="54"/>
+      <c r="B229" s="42"/>
+      <c r="AA229" s="43"/>
     </row>
     <row r="230" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B230" s="53"/>
-      <c r="AA230" s="54"/>
+      <c r="B230" s="42"/>
+      <c r="AA230" s="43"/>
     </row>
     <row r="231" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B231" s="53"/>
-      <c r="AA231" s="54"/>
+      <c r="B231" s="42"/>
+      <c r="AA231" s="43"/>
     </row>
     <row r="232" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B232" s="53"/>
-      <c r="AA232" s="54"/>
+      <c r="B232" s="42"/>
+      <c r="AA232" s="43"/>
     </row>
     <row r="233" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B233" s="53"/>
-      <c r="AA233" s="54"/>
+      <c r="B233" s="42"/>
+      <c r="AA233" s="43"/>
     </row>
     <row r="234" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B234" s="53"/>
-      <c r="AA234" s="54"/>
+      <c r="B234" s="42"/>
+      <c r="AA234" s="43"/>
     </row>
     <row r="235" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B235" s="53"/>
-      <c r="AA235" s="54"/>
+      <c r="B235" s="42"/>
+      <c r="AA235" s="43"/>
     </row>
     <row r="236" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B236" s="53"/>
-      <c r="AA236" s="54"/>
+      <c r="B236" s="42"/>
+      <c r="AA236" s="43"/>
     </row>
     <row r="237" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B237" s="53"/>
-      <c r="AA237" s="54"/>
+      <c r="B237" s="42"/>
+      <c r="AA237" s="43"/>
     </row>
     <row r="238" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B238" s="53"/>
-      <c r="AA238" s="54"/>
+      <c r="B238" s="42"/>
+      <c r="AA238" s="43"/>
     </row>
     <row r="239" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B239" s="53"/>
-      <c r="AA239" s="54"/>
+      <c r="B239" s="42"/>
+      <c r="AA239" s="43"/>
     </row>
     <row r="240" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B240" s="53"/>
-      <c r="AA240" s="54"/>
+      <c r="B240" s="42"/>
+      <c r="AA240" s="43"/>
     </row>
     <row r="241" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B241" s="53"/>
-      <c r="AA241" s="54"/>
+      <c r="B241" s="42"/>
+      <c r="AA241" s="43"/>
     </row>
     <row r="242" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B242" s="53"/>
-      <c r="AA242" s="54"/>
+      <c r="B242" s="42"/>
+      <c r="AA242" s="43"/>
     </row>
     <row r="243" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B243" s="53"/>
-      <c r="AA243" s="54"/>
+      <c r="B243" s="42"/>
+      <c r="AA243" s="43"/>
     </row>
     <row r="244" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B244" s="53"/>
-      <c r="AA244" s="54"/>
+      <c r="B244" s="42"/>
+      <c r="AA244" s="43"/>
     </row>
     <row r="245" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B245" s="53"/>
-      <c r="AA245" s="54"/>
+      <c r="B245" s="42"/>
+      <c r="AA245" s="43"/>
     </row>
     <row r="246" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B246" s="53"/>
-      <c r="AA246" s="54"/>
+      <c r="B246" s="42"/>
+      <c r="AA246" s="43"/>
     </row>
     <row r="247" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B247" s="53"/>
-      <c r="AA247" s="54"/>
+      <c r="B247" s="42"/>
+      <c r="AA247" s="43"/>
     </row>
     <row r="248" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B248" s="53"/>
-      <c r="AA248" s="54"/>
+      <c r="B248" s="42"/>
+      <c r="AA248" s="43"/>
     </row>
     <row r="249" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B249" s="53"/>
-      <c r="AA249" s="54"/>
+      <c r="B249" s="42"/>
+      <c r="AA249" s="43"/>
     </row>
     <row r="250" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B250" s="53"/>
-      <c r="AA250" s="54"/>
+      <c r="B250" s="42"/>
+      <c r="AA250" s="43"/>
     </row>
     <row r="251" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B251" s="53"/>
-      <c r="AA251" s="54"/>
+      <c r="B251" s="42"/>
+      <c r="AA251" s="43"/>
     </row>
     <row r="252" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B252" s="53"/>
-      <c r="AA252" s="54"/>
+      <c r="B252" s="42"/>
+      <c r="AA252" s="43"/>
     </row>
     <row r="253" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B253" s="53"/>
-      <c r="AA253" s="54"/>
+      <c r="B253" s="42"/>
+      <c r="AA253" s="43"/>
     </row>
     <row r="254" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B254" s="53"/>
-      <c r="AA254" s="54"/>
+      <c r="B254" s="42"/>
+      <c r="AA254" s="43"/>
     </row>
     <row r="255" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B255" s="53"/>
-      <c r="AA255" s="54"/>
+      <c r="B255" s="42"/>
+      <c r="AA255" s="43"/>
     </row>
     <row r="256" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B256" s="53"/>
-      <c r="AA256" s="54"/>
+      <c r="B256" s="42"/>
+      <c r="AA256" s="43"/>
     </row>
     <row r="257" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B257" s="53"/>
-      <c r="AA257" s="54"/>
+      <c r="B257" s="42"/>
+      <c r="AA257" s="43"/>
     </row>
     <row r="258" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B258" s="53"/>
-      <c r="AA258" s="54"/>
+      <c r="B258" s="42"/>
+      <c r="AA258" s="43"/>
     </row>
     <row r="259" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B259" s="53"/>
-      <c r="AA259" s="54"/>
+      <c r="B259" s="42"/>
+      <c r="AA259" s="43"/>
     </row>
     <row r="260" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B260" s="53"/>
-      <c r="AA260" s="54"/>
+      <c r="B260" s="42"/>
+      <c r="AA260" s="43"/>
     </row>
     <row r="261" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B261" s="53"/>
-      <c r="AA261" s="54"/>
+      <c r="B261" s="42"/>
+      <c r="AA261" s="43"/>
     </row>
     <row r="262" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B262" s="53"/>
-      <c r="AA262" s="54"/>
+      <c r="B262" s="42"/>
+      <c r="AA262" s="43"/>
     </row>
     <row r="263" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B263" s="53"/>
-      <c r="AA263" s="54"/>
+      <c r="B263" s="42"/>
+      <c r="AA263" s="43"/>
     </row>
     <row r="264" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B264" s="53"/>
-      <c r="AA264" s="54"/>
+      <c r="B264" s="42"/>
+      <c r="AA264" s="43"/>
     </row>
     <row r="265" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B265" s="53"/>
-      <c r="AA265" s="54"/>
+      <c r="B265" s="42"/>
+      <c r="AA265" s="43"/>
     </row>
     <row r="266" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B266" s="53"/>
-      <c r="AA266" s="54"/>
+      <c r="B266" s="42"/>
+      <c r="AA266" s="43"/>
     </row>
     <row r="267" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B267" s="53"/>
-      <c r="AA267" s="54"/>
+      <c r="B267" s="42"/>
+      <c r="AA267" s="43"/>
     </row>
     <row r="268" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B268" s="53"/>
-      <c r="AA268" s="54"/>
+      <c r="B268" s="42"/>
+      <c r="AA268" s="43"/>
     </row>
     <row r="269" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B269" s="53"/>
-      <c r="AA269" s="54"/>
+      <c r="B269" s="42"/>
+      <c r="AA269" s="43"/>
     </row>
     <row r="270" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B270" s="53"/>
-      <c r="AA270" s="54"/>
+      <c r="B270" s="42"/>
+      <c r="AA270" s="43"/>
     </row>
     <row r="271" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B271" s="53"/>
-      <c r="AA271" s="54"/>
+      <c r="B271" s="42"/>
+      <c r="AA271" s="43"/>
     </row>
     <row r="272" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B272" s="53"/>
-      <c r="AA272" s="54"/>
+      <c r="B272" s="42"/>
+      <c r="AA272" s="43"/>
     </row>
     <row r="273" spans="2:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B273" s="53"/>
-      <c r="AA273" s="54"/>
+      <c r="B273" s="42"/>
+      <c r="AA273" s="43"/>
     </row>
     <row r="274" spans="2:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B274" s="53"/>
-      <c r="AA274" s="54"/>
+      <c r="B274" s="42"/>
+      <c r="AA274" s="43"/>
     </row>
     <row r="275" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B275" s="53"/>
-      <c r="AA275" s="54"/>
+      <c r="B275" s="42"/>
+      <c r="AA275" s="43"/>
     </row>
     <row r="276" spans="2:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B276" s="53"/>
-      <c r="AA276" s="54"/>
+      <c r="B276" s="42"/>
+      <c r="AA276" s="43"/>
     </row>
     <row r="277" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B277" s="53"/>
-      <c r="AA277" s="54"/>
+      <c r="B277" s="42"/>
+      <c r="AA277" s="43"/>
     </row>
     <row r="278" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B278" s="53"/>
-      <c r="AA278" s="54"/>
+      <c r="B278" s="42"/>
+      <c r="AA278" s="43"/>
     </row>
     <row r="279" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B279" s="53"/>
-      <c r="AA279" s="54"/>
+      <c r="B279" s="42"/>
+      <c r="AA279" s="43"/>
     </row>
     <row r="280" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B280" s="53"/>
-      <c r="AA280" s="54"/>
+      <c r="B280" s="42"/>
+      <c r="AA280" s="43"/>
     </row>
     <row r="281" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B281" s="53"/>
-      <c r="AA281" s="54"/>
+      <c r="B281" s="42"/>
+      <c r="AA281" s="43"/>
     </row>
     <row r="282" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B282" s="53"/>
-      <c r="AA282" s="54"/>
+      <c r="B282" s="42"/>
+      <c r="AA282" s="43"/>
     </row>
     <row r="283" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B283" s="53"/>
-      <c r="AA283" s="54"/>
+      <c r="B283" s="42"/>
+      <c r="AA283" s="43"/>
     </row>
     <row r="284" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B284" s="53"/>
-      <c r="AA284" s="54"/>
+      <c r="B284" s="42"/>
+      <c r="AA284" s="43"/>
     </row>
     <row r="285" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B285" s="53"/>
-      <c r="AA285" s="54"/>
+      <c r="B285" s="42"/>
+      <c r="AA285" s="43"/>
     </row>
     <row r="286" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B286" s="53"/>
-      <c r="AA286" s="54"/>
+      <c r="B286" s="42"/>
+      <c r="AA286" s="43"/>
     </row>
     <row r="287" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B287" s="53"/>
-      <c r="AA287" s="54"/>
+      <c r="B287" s="42"/>
+      <c r="AA287" s="43"/>
     </row>
     <row r="288" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B288" s="53"/>
-      <c r="AA288" s="54"/>
+      <c r="B288" s="42"/>
+      <c r="AA288" s="43"/>
     </row>
     <row r="289" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B289" s="53"/>
-      <c r="AA289" s="54"/>
+      <c r="B289" s="42"/>
+      <c r="AA289" s="43"/>
     </row>
     <row r="290" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B290" s="53"/>
-      <c r="AA290" s="54"/>
+      <c r="B290" s="42"/>
+      <c r="AA290" s="43"/>
     </row>
     <row r="291" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B291" s="53"/>
-      <c r="AA291" s="54"/>
+      <c r="B291" s="42"/>
+      <c r="AA291" s="43"/>
     </row>
     <row r="292" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B292" s="53"/>
-      <c r="AA292" s="54"/>
+      <c r="B292" s="42"/>
+      <c r="AA292" s="43"/>
     </row>
     <row r="293" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B293" s="53"/>
-      <c r="AA293" s="54"/>
+      <c r="B293" s="42"/>
+      <c r="AA293" s="43"/>
     </row>
     <row r="294" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B294" s="53"/>
-      <c r="AA294" s="54"/>
+      <c r="B294" s="42"/>
+      <c r="AA294" s="43"/>
     </row>
     <row r="295" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B295" s="53"/>
-      <c r="AA295" s="54"/>
+      <c r="B295" s="42"/>
+      <c r="AA295" s="43"/>
     </row>
     <row r="296" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B296" s="53"/>
-      <c r="AA296" s="54"/>
+      <c r="B296" s="42"/>
+      <c r="AA296" s="43"/>
     </row>
     <row r="297" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B297" s="53"/>
-      <c r="AA297" s="54"/>
+      <c r="B297" s="42"/>
+      <c r="AA297" s="43"/>
     </row>
     <row r="298" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B298" s="53"/>
-      <c r="AA298" s="54"/>
+      <c r="B298" s="42"/>
+      <c r="AA298" s="43"/>
     </row>
     <row r="299" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B299" s="53"/>
-      <c r="AA299" s="54"/>
+      <c r="B299" s="42"/>
+      <c r="AA299" s="43"/>
     </row>
     <row r="300" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B300" s="53"/>
-      <c r="AA300" s="54"/>
+      <c r="B300" s="42"/>
+      <c r="AA300" s="43"/>
     </row>
     <row r="301" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B301" s="53"/>
-      <c r="AA301" s="54"/>
+      <c r="B301" s="42"/>
+      <c r="AA301" s="43"/>
     </row>
     <row r="302" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B302" s="53"/>
-      <c r="AA302" s="54"/>
+      <c r="B302" s="42"/>
+      <c r="AA302" s="43"/>
     </row>
     <row r="303" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B303" s="53"/>
-      <c r="AA303" s="54"/>
+      <c r="B303" s="42"/>
+      <c r="AA303" s="43"/>
     </row>
     <row r="304" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B304" s="53"/>
-      <c r="AA304" s="54"/>
+      <c r="B304" s="42"/>
+      <c r="AA304" s="43"/>
     </row>
     <row r="305" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B305" s="53"/>
-      <c r="AA305" s="54"/>
+      <c r="B305" s="42"/>
+      <c r="AA305" s="43"/>
     </row>
     <row r="306" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B306" s="53"/>
-      <c r="AA306" s="54"/>
+      <c r="B306" s="42"/>
+      <c r="AA306" s="43"/>
     </row>
     <row r="307" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B307" s="53"/>
-      <c r="AA307" s="54"/>
+      <c r="B307" s="42"/>
+      <c r="AA307" s="43"/>
     </row>
     <row r="308" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B308" s="53"/>
-      <c r="AA308" s="54"/>
+      <c r="B308" s="42"/>
+      <c r="AA308" s="43"/>
     </row>
     <row r="309" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B309" s="53"/>
-      <c r="AA309" s="54"/>
+      <c r="B309" s="42"/>
+      <c r="AA309" s="43"/>
     </row>
     <row r="310" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B310" s="53"/>
-      <c r="AA310" s="54"/>
+      <c r="B310" s="42"/>
+      <c r="AA310" s="43"/>
     </row>
     <row r="311" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B311" s="53"/>
-      <c r="AA311" s="54"/>
+      <c r="B311" s="42"/>
+      <c r="AA311" s="43"/>
     </row>
     <row r="312" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B312" s="53"/>
-      <c r="AA312" s="54"/>
+      <c r="B312" s="42"/>
+      <c r="AA312" s="43"/>
     </row>
     <row r="313" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B313" s="53"/>
-      <c r="AA313" s="54"/>
+      <c r="B313" s="42"/>
+      <c r="AA313" s="43"/>
     </row>
     <row r="314" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B314" s="53"/>
-      <c r="AA314" s="54"/>
+      <c r="B314" s="42"/>
+      <c r="AA314" s="43"/>
     </row>
     <row r="315" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B315" s="53"/>
-      <c r="AA315" s="54"/>
+      <c r="B315" s="42"/>
+      <c r="AA315" s="43"/>
     </row>
     <row r="316" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B316" s="53"/>
-      <c r="AA316" s="54"/>
+      <c r="B316" s="42"/>
+      <c r="AA316" s="43"/>
     </row>
     <row r="317" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B317" s="53"/>
-      <c r="AA317" s="54"/>
+      <c r="B317" s="42"/>
+      <c r="AA317" s="43"/>
     </row>
     <row r="318" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B318" s="53"/>
-      <c r="AA318" s="54"/>
+      <c r="B318" s="42"/>
+      <c r="AA318" s="43"/>
     </row>
     <row r="319" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B319" s="53"/>
-      <c r="AA319" s="54"/>
+      <c r="B319" s="42"/>
+      <c r="AA319" s="43"/>
     </row>
     <row r="320" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B320" s="53"/>
-      <c r="AA320" s="54"/>
+      <c r="B320" s="42"/>
+      <c r="AA320" s="43"/>
     </row>
     <row r="321" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B321" s="53"/>
-      <c r="AA321" s="54"/>
+      <c r="B321" s="42"/>
+      <c r="AA321" s="43"/>
     </row>
     <row r="322" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B322" s="53"/>
-      <c r="AA322" s="54"/>
+      <c r="B322" s="42"/>
+      <c r="AA322" s="43"/>
     </row>
     <row r="323" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B323" s="53"/>
-      <c r="AA323" s="54"/>
+      <c r="B323" s="42"/>
+      <c r="AA323" s="43"/>
     </row>
     <row r="324" spans="2:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B324" s="53"/>
-      <c r="AA324" s="54"/>
+      <c r="B324" s="42"/>
+      <c r="AA324" s="43"/>
     </row>
     <row r="325" spans="2:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B325" s="53"/>
-      <c r="AA325" s="54"/>
+      <c r="B325" s="42"/>
+      <c r="AA325" s="43"/>
     </row>
     <row r="326" spans="2:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B326" s="53"/>
-      <c r="AA326" s="54"/>
+      <c r="B326" s="42"/>
+      <c r="AA326" s="43"/>
     </row>
     <row r="327" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B327" s="53"/>
-      <c r="AA327" s="54"/>
+      <c r="B327" s="42"/>
+      <c r="AA327" s="43"/>
     </row>
     <row r="328" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B328" s="53"/>
-      <c r="AA328" s="54"/>
+      <c r="B328" s="42"/>
+      <c r="AA328" s="43"/>
     </row>
     <row r="329" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B329" s="53"/>
-      <c r="AA329" s="54"/>
+      <c r="B329" s="42"/>
+      <c r="AA329" s="43"/>
     </row>
     <row r="330" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B330" s="53"/>
-      <c r="AA330" s="54"/>
+      <c r="B330" s="42"/>
+      <c r="AA330" s="43"/>
     </row>
     <row r="331" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B331" s="53"/>
-      <c r="AA331" s="54"/>
+      <c r="B331" s="42"/>
+      <c r="AA331" s="43"/>
     </row>
     <row r="332" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B332" s="53"/>
-      <c r="AA332" s="54"/>
+      <c r="B332" s="42"/>
+      <c r="AA332" s="43"/>
     </row>
     <row r="333" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B333" s="53"/>
-      <c r="AA333" s="54"/>
+      <c r="B333" s="42"/>
+      <c r="AA333" s="43"/>
     </row>
     <row r="334" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B334" s="53"/>
-      <c r="AA334" s="54"/>
+      <c r="B334" s="42"/>
+      <c r="AA334" s="43"/>
     </row>
     <row r="335" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B335" s="53"/>
-      <c r="AA335" s="54"/>
+      <c r="B335" s="42"/>
+      <c r="AA335" s="43"/>
     </row>
     <row r="336" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B336" s="53"/>
-      <c r="AA336" s="54"/>
+      <c r="B336" s="42"/>
+      <c r="AA336" s="43"/>
     </row>
     <row r="337" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B337" s="53"/>
-      <c r="AA337" s="54"/>
+      <c r="B337" s="42"/>
+      <c r="AA337" s="43"/>
     </row>
     <row r="338" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B338" s="53"/>
-      <c r="AA338" s="54"/>
+      <c r="B338" s="42"/>
+      <c r="AA338" s="43"/>
     </row>
     <row r="339" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B339" s="53"/>
-      <c r="AA339" s="54"/>
+      <c r="B339" s="42"/>
+      <c r="AA339" s="43"/>
     </row>
     <row r="340" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B340" s="53"/>
-      <c r="AA340" s="54"/>
+      <c r="B340" s="42"/>
+      <c r="AA340" s="43"/>
     </row>
     <row r="341" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B341" s="53"/>
-      <c r="AA341" s="54"/>
+      <c r="B341" s="42"/>
+      <c r="AA341" s="43"/>
     </row>
     <row r="342" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B342" s="53"/>
-      <c r="AA342" s="54"/>
+      <c r="B342" s="42"/>
+      <c r="AA342" s="43"/>
     </row>
     <row r="343" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B343" s="53"/>
-      <c r="AA343" s="54"/>
+      <c r="B343" s="42"/>
+      <c r="AA343" s="43"/>
     </row>
     <row r="344" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B344" s="53"/>
-      <c r="AA344" s="54"/>
+      <c r="B344" s="42"/>
+      <c r="AA344" s="43"/>
     </row>
     <row r="345" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B345" s="53"/>
-      <c r="AA345" s="54"/>
+      <c r="B345" s="42"/>
+      <c r="AA345" s="43"/>
     </row>
     <row r="346" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B346" s="53"/>
-      <c r="AA346" s="54"/>
+      <c r="B346" s="42"/>
+      <c r="AA346" s="43"/>
     </row>
     <row r="347" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B347" s="53"/>
-      <c r="AA347" s="54"/>
+      <c r="B347" s="42"/>
+      <c r="AA347" s="43"/>
     </row>
     <row r="348" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B348" s="53"/>
-      <c r="AA348" s="54"/>
+      <c r="B348" s="42"/>
+      <c r="AA348" s="43"/>
     </row>
     <row r="349" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B349" s="53"/>
-      <c r="AA349" s="54"/>
+      <c r="B349" s="42"/>
+      <c r="AA349" s="43"/>
     </row>
     <row r="350" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B350" s="53"/>
-      <c r="AA350" s="54"/>
+      <c r="B350" s="42"/>
+      <c r="AA350" s="43"/>
     </row>
     <row r="351" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B351" s="53"/>
-      <c r="AA351" s="54"/>
+      <c r="B351" s="42"/>
+      <c r="AA351" s="43"/>
     </row>
     <row r="352" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B352" s="53"/>
-      <c r="AA352" s="54"/>
+      <c r="B352" s="42"/>
+      <c r="AA352" s="43"/>
     </row>
     <row r="353" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B353" s="53"/>
-      <c r="AA353" s="54"/>
+      <c r="B353" s="42"/>
+      <c r="AA353" s="43"/>
     </row>
     <row r="354" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B354" s="53"/>
-      <c r="AA354" s="54"/>
+      <c r="B354" s="42"/>
+      <c r="AA354" s="43"/>
     </row>
     <row r="355" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B355" s="53"/>
-      <c r="AA355" s="54"/>
+      <c r="B355" s="42"/>
+      <c r="AA355" s="43"/>
     </row>
     <row r="356" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B356" s="53"/>
-      <c r="AA356" s="54"/>
+      <c r="B356" s="42"/>
+      <c r="AA356" s="43"/>
     </row>
     <row r="357" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B357" s="53"/>
-      <c r="AA357" s="54"/>
+      <c r="B357" s="42"/>
+      <c r="AA357" s="43"/>
     </row>
     <row r="358" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B358" s="53"/>
-      <c r="AA358" s="54"/>
+      <c r="B358" s="42"/>
+      <c r="AA358" s="43"/>
     </row>
     <row r="359" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B359" s="53"/>
-      <c r="AA359" s="54"/>
+      <c r="B359" s="42"/>
+      <c r="AA359" s="43"/>
     </row>
     <row r="360" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B360" s="53"/>
-      <c r="AA360" s="54"/>
+      <c r="B360" s="42"/>
+      <c r="AA360" s="43"/>
     </row>
     <row r="361" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B361" s="53"/>
-      <c r="AA361" s="54"/>
+      <c r="B361" s="42"/>
+      <c r="AA361" s="43"/>
     </row>
     <row r="362" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B362" s="53"/>
-      <c r="AA362" s="54"/>
+      <c r="B362" s="42"/>
+      <c r="AA362" s="43"/>
     </row>
     <row r="363" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B363" s="53"/>
-      <c r="AA363" s="54"/>
+      <c r="B363" s="42"/>
+      <c r="AA363" s="43"/>
     </row>
     <row r="364" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B364" s="53"/>
-      <c r="AA364" s="54"/>
+      <c r="B364" s="42"/>
+      <c r="AA364" s="43"/>
     </row>
     <row r="365" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B365" s="53"/>
-      <c r="AA365" s="54"/>
+      <c r="B365" s="42"/>
+      <c r="AA365" s="43"/>
     </row>
     <row r="366" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B366" s="53"/>
-      <c r="AA366" s="54"/>
+      <c r="B366" s="42"/>
+      <c r="AA366" s="43"/>
     </row>
     <row r="367" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B367" s="53"/>
-      <c r="AA367" s="54"/>
+      <c r="B367" s="42"/>
+      <c r="AA367" s="43"/>
     </row>
     <row r="368" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B368" s="53"/>
-      <c r="AA368" s="54"/>
+      <c r="B368" s="42"/>
+      <c r="AA368" s="43"/>
     </row>
     <row r="369" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B369" s="53"/>
-      <c r="AA369" s="54"/>
+      <c r="B369" s="42"/>
+      <c r="AA369" s="43"/>
     </row>
     <row r="370" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B370" s="53"/>
-      <c r="AA370" s="54"/>
+      <c r="B370" s="42"/>
+      <c r="AA370" s="43"/>
     </row>
     <row r="371" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B371" s="53"/>
-      <c r="AA371" s="54"/>
+      <c r="B371" s="42"/>
+      <c r="AA371" s="43"/>
     </row>
     <row r="372" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B372" s="53"/>
-      <c r="AA372" s="54"/>
+      <c r="B372" s="42"/>
+      <c r="AA372" s="43"/>
     </row>
     <row r="373" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B373" s="53"/>
-      <c r="AA373" s="54"/>
+      <c r="B373" s="42"/>
+      <c r="AA373" s="43"/>
     </row>
     <row r="374" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B374" s="53"/>
-      <c r="AA374" s="54"/>
+      <c r="B374" s="42"/>
+      <c r="AA374" s="43"/>
     </row>
     <row r="375" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B375" s="53"/>
-      <c r="AA375" s="54"/>
+      <c r="B375" s="42"/>
+      <c r="AA375" s="43"/>
     </row>
     <row r="376" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B376" s="53"/>
-      <c r="AA376" s="54"/>
+      <c r="B376" s="42"/>
+      <c r="AA376" s="43"/>
     </row>
     <row r="377" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B377" s="53"/>
-      <c r="AA377" s="54"/>
+      <c r="B377" s="42"/>
+      <c r="AA377" s="43"/>
     </row>
     <row r="378" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B378" s="53"/>
-      <c r="AA378" s="54"/>
+      <c r="B378" s="42"/>
+      <c r="AA378" s="43"/>
     </row>
     <row r="379" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B379" s="53"/>
-      <c r="AA379" s="54"/>
+      <c r="B379" s="42"/>
+      <c r="AA379" s="43"/>
     </row>
     <row r="380" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B380" s="53"/>
-      <c r="AA380" s="54"/>
+      <c r="B380" s="42"/>
+      <c r="AA380" s="43"/>
     </row>
     <row r="381" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B381" s="53"/>
-      <c r="AA381" s="54"/>
+      <c r="B381" s="42"/>
+      <c r="AA381" s="43"/>
     </row>
     <row r="382" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B382" s="53"/>
-      <c r="AA382" s="54"/>
+      <c r="B382" s="42"/>
+      <c r="AA382" s="43"/>
     </row>
     <row r="383" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B383" s="53"/>
-      <c r="AA383" s="54"/>
+      <c r="B383" s="42"/>
+      <c r="AA383" s="43"/>
     </row>
     <row r="384" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B384" s="53"/>
-      <c r="AA384" s="54"/>
+      <c r="B384" s="42"/>
+      <c r="AA384" s="43"/>
     </row>
     <row r="385" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B385" s="53"/>
-      <c r="AA385" s="54"/>
+      <c r="B385" s="42"/>
+      <c r="AA385" s="43"/>
     </row>
     <row r="386" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B386" s="53"/>
-      <c r="AA386" s="54"/>
+      <c r="B386" s="42"/>
+      <c r="AA386" s="43"/>
     </row>
     <row r="387" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B387" s="53"/>
-      <c r="AA387" s="54"/>
+      <c r="B387" s="42"/>
+      <c r="AA387" s="43"/>
     </row>
     <row r="388" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B388" s="53"/>
-      <c r="AA388" s="54"/>
+      <c r="B388" s="42"/>
+      <c r="AA388" s="43"/>
     </row>
     <row r="389" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B389" s="53"/>
-      <c r="AA389" s="54"/>
+      <c r="B389" s="42"/>
+      <c r="AA389" s="43"/>
     </row>
     <row r="390" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B390" s="53"/>
-      <c r="AA390" s="54"/>
+      <c r="B390" s="42"/>
+      <c r="AA390" s="43"/>
     </row>
     <row r="391" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B391" s="53"/>
-      <c r="AA391" s="54"/>
+      <c r="B391" s="42"/>
+      <c r="AA391" s="43"/>
     </row>
     <row r="392" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B392" s="53"/>
-      <c r="AA392" s="54"/>
+      <c r="B392" s="42"/>
+      <c r="AA392" s="43"/>
     </row>
     <row r="393" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B393" s="53"/>
-      <c r="AA393" s="54"/>
+      <c r="B393" s="42"/>
+      <c r="AA393" s="43"/>
     </row>
     <row r="394" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B394" s="53"/>
-      <c r="AA394" s="54"/>
+      <c r="B394" s="42"/>
+      <c r="AA394" s="43"/>
     </row>
     <row r="395" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B395" s="53"/>
-      <c r="AA395" s="54"/>
+      <c r="B395" s="42"/>
+      <c r="AA395" s="43"/>
     </row>
     <row r="396" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B396" s="53"/>
-      <c r="AA396" s="54"/>
+      <c r="B396" s="42"/>
+      <c r="AA396" s="43"/>
     </row>
     <row r="397" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B397" s="53"/>
-      <c r="AA397" s="54"/>
+      <c r="B397" s="42"/>
+      <c r="AA397" s="43"/>
     </row>
     <row r="398" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B398" s="53"/>
-      <c r="AA398" s="54"/>
+      <c r="B398" s="42"/>
+      <c r="AA398" s="43"/>
     </row>
     <row r="399" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B399" s="53"/>
-      <c r="AA399" s="54"/>
+      <c r="B399" s="42"/>
+      <c r="AA399" s="43"/>
     </row>
     <row r="400" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B400" s="53"/>
-      <c r="AA400" s="54"/>
+      <c r="B400" s="42"/>
+      <c r="AA400" s="43"/>
     </row>
     <row r="401" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B401" s="53"/>
-      <c r="AA401" s="54"/>
+      <c r="B401" s="42"/>
+      <c r="AA401" s="43"/>
     </row>
     <row r="402" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B402" s="53"/>
-      <c r="AA402" s="54"/>
+      <c r="B402" s="42"/>
+      <c r="AA402" s="43"/>
     </row>
     <row r="403" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B403" s="53"/>
-      <c r="AA403" s="54"/>
+      <c r="B403" s="42"/>
+      <c r="AA403" s="43"/>
     </row>
     <row r="404" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B404" s="53"/>
-      <c r="AA404" s="54"/>
+      <c r="B404" s="42"/>
+      <c r="AA404" s="43"/>
     </row>
     <row r="405" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B405" s="53"/>
-      <c r="AA405" s="54"/>
+      <c r="B405" s="42"/>
+      <c r="AA405" s="43"/>
     </row>
     <row r="406" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B406" s="53"/>
-      <c r="AA406" s="54"/>
+      <c r="B406" s="42"/>
+      <c r="AA406" s="43"/>
     </row>
     <row r="407" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B407" s="53"/>
-      <c r="AA407" s="54"/>
+      <c r="B407" s="42"/>
+      <c r="AA407" s="43"/>
     </row>
     <row r="408" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B408" s="53"/>
-      <c r="AA408" s="54"/>
+      <c r="B408" s="42"/>
+      <c r="AA408" s="43"/>
     </row>
     <row r="409" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B409" s="53"/>
-      <c r="AA409" s="54"/>
+      <c r="B409" s="42"/>
+      <c r="AA409" s="43"/>
     </row>
     <row r="410" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B410" s="53"/>
-      <c r="AA410" s="54"/>
+      <c r="B410" s="42"/>
+      <c r="AA410" s="43"/>
     </row>
     <row r="411" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B411" s="53"/>
-      <c r="AA411" s="54"/>
+      <c r="B411" s="42"/>
+      <c r="AA411" s="43"/>
     </row>
     <row r="412" spans="2:27" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B412" s="53"/>
-      <c r="AA412" s="54"/>
+      <c r="B412" s="42"/>
+      <c r="AA412" s="43"/>
     </row>
     <row r="413" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B413" s="53"/>
-      <c r="AA413" s="54"/>
+      <c r="B413" s="42"/>
+      <c r="AA413" s="43"/>
     </row>
     <row r="414" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B414" s="53"/>
-      <c r="AA414" s="54"/>
+      <c r="B414" s="42"/>
+      <c r="AA414" s="43"/>
     </row>
     <row r="415" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B415" s="53"/>
-      <c r="AA415" s="54"/>
+      <c r="B415" s="42"/>
+      <c r="AA415" s="43"/>
     </row>
     <row r="416" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B416" s="53"/>
-      <c r="AA416" s="54"/>
+      <c r="B416" s="42"/>
+      <c r="AA416" s="43"/>
     </row>
     <row r="417" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B417" s="53"/>
-      <c r="AA417" s="54"/>
+      <c r="B417" s="42"/>
+      <c r="AA417" s="43"/>
     </row>
     <row r="418" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B418" s="53"/>
-      <c r="AA418" s="54"/>
+      <c r="B418" s="42"/>
+      <c r="AA418" s="43"/>
     </row>
     <row r="419" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B419" s="55"/>
-      <c r="C419" s="56"/>
-      <c r="D419" s="56"/>
-      <c r="E419" s="56"/>
-      <c r="F419" s="56"/>
-      <c r="G419" s="56"/>
-      <c r="H419" s="56"/>
-      <c r="I419" s="56"/>
-      <c r="J419" s="56"/>
-      <c r="K419" s="56"/>
-      <c r="L419" s="56"/>
-      <c r="M419" s="56"/>
-      <c r="N419" s="56"/>
-      <c r="O419" s="56"/>
-      <c r="P419" s="56"/>
-      <c r="Q419" s="56"/>
-      <c r="R419" s="56"/>
-      <c r="S419" s="56"/>
-      <c r="T419" s="56"/>
-      <c r="U419" s="56"/>
-      <c r="V419" s="56"/>
-      <c r="W419" s="65"/>
-      <c r="X419" s="65"/>
-      <c r="Y419" s="56"/>
-      <c r="Z419" s="56"/>
-      <c r="AA419" s="57"/>
+      <c r="B419" s="44"/>
+      <c r="C419" s="45"/>
+      <c r="D419" s="45"/>
+      <c r="E419" s="45"/>
+      <c r="F419" s="45"/>
+      <c r="G419" s="45"/>
+      <c r="H419" s="45"/>
+      <c r="I419" s="45"/>
+      <c r="J419" s="45"/>
+      <c r="K419" s="45"/>
+      <c r="L419" s="45"/>
+      <c r="M419" s="45"/>
+      <c r="N419" s="45"/>
+      <c r="O419" s="45"/>
+      <c r="P419" s="45"/>
+      <c r="Q419" s="45"/>
+      <c r="R419" s="45"/>
+      <c r="S419" s="45"/>
+      <c r="T419" s="45"/>
+      <c r="U419" s="45"/>
+      <c r="V419" s="45"/>
+      <c r="W419" s="54"/>
+      <c r="X419" s="54"/>
+      <c r="Y419" s="45"/>
+      <c r="Z419" s="45"/>
+      <c r="AA419" s="46"/>
     </row>
   </sheetData>
   <pageMargins left="0.78740157480314965" right="0.78740157480314965" top="0.55118110236220474" bottom="0.98425196850393704" header="0" footer="0"/>

</xml_diff>